<commit_message>
produktjakt Carashell: hjulskydden 4-pack (K0068) på Axels fråga — batch 17, sida v32, ark ombyggt
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jBJVGuyny8S3j2XPSM26Z
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-29-carashell/Leverantorsoffert-2026-09-29-carashell.xlsx
+++ b/produktjakt/korningar/2026-09-29-carashell/Leverantorsoffert-2026-09-29-carashell.xlsx
@@ -866,7 +866,7 @@
       <row>56</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1533525" cy="1600200"/>
+    <ext cx="1600200" cy="1600200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="14" name="Image 14" descr="Picture"/>
@@ -891,7 +891,7 @@
       <row>60</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1600200" cy="1600200"/>
+    <ext cx="1533525" cy="1600200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -924,6 +924,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1600200" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1137,7 +1162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU68"/>
+  <dimension ref="A1:AU72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="71" min="1" max="1"/>
@@ -1172,7 +1197,7 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="71">
       <c r="A1" s="1" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AP1" s="1" t="n"/>
       <c r="AQ1" s="1" t="n"/>
@@ -2284,12 +2309,12 @@
       <c r="A25" s="10" t="n"/>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>Bakdörrsgardinerna Ducato, 2 delar</t>
+          <t>Hjulskydden 4-pack, silver 19–36 tum</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $26.19. Vår räkning: landad ca 379 kr, tänkt butikspris 1199 kr. Originaltitel: Bakdörrsgardinerna Ducato, 2 delar</t>
+          <t>AliExpress: US $24.49. Vår räkning: landad ca 355 kr, tänkt butikspris 599 kr. Originaltitel: Hjulskydden 4-pack, silver 19–36 tum</t>
         </is>
       </c>
       <c r="H25" s="13" t="n"/>
@@ -2304,7 +2329,7 @@
       <c r="M25" s="14" t="n"/>
       <c r="N25" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010569162335.html</t>
+          <t>https://www.aliexpress.com/item/1005005932851254.html</t>
         </is>
       </c>
       <c r="Q25" s="18" t="n"/>
@@ -2454,12 +2479,12 @@
       <c r="A29" s="10" t="n"/>
       <c r="D29" s="18" t="inlineStr">
         <is>
-          <t>Husbilens spegelhuvar i par, Ducato</t>
+          <t>Bakdörrsgardinerna Ducato, 2 delar</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $28.59. Vår räkning: landad ca 414 kr, tänkt butikspris 699 kr. Originaltitel: Husbilens spegelhuvar i par, Ducato</t>
+          <t>AliExpress: US $26.19. Vår räkning: landad ca 379 kr, tänkt butikspris 1199 kr. Originaltitel: Bakdörrsgardinerna Ducato, 2 delar</t>
         </is>
       </c>
       <c r="H29" s="13" t="n"/>
@@ -2474,7 +2499,7 @@
       <c r="M29" s="14" t="n"/>
       <c r="N29" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010581700454.html</t>
+          <t>https://www.aliexpress.com/item/1005010569162335.html</t>
         </is>
       </c>
       <c r="Q29" s="18" t="n"/>
@@ -2624,12 +2649,12 @@
       <c r="A33" s="10" t="n"/>
       <c r="D33" s="18" t="inlineStr">
         <is>
-          <t>Vindavvisarna till Ducato-hytten, par</t>
+          <t>Husbilens spegelhuvar i par, Ducato</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $24.09. Vår räkning: landad ca 348 kr, tänkt butikspris 649 kr. Originaltitel: Vindavvisarna till Ducato-hytten, par</t>
+          <t>AliExpress: US $28.59. Vår räkning: landad ca 414 kr, tänkt butikspris 699 kr. Originaltitel: Husbilens spegelhuvar i par, Ducato</t>
         </is>
       </c>
       <c r="H33" s="13" t="n"/>
@@ -2644,7 +2669,7 @@
       <c r="M33" s="14" t="n"/>
       <c r="N33" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012880104542.html</t>
+          <t>https://www.aliexpress.com/item/1005010581700454.html</t>
         </is>
       </c>
       <c r="Q33" s="18" t="n"/>
@@ -2794,12 +2819,12 @@
       <c r="A37" s="10" t="n"/>
       <c r="D37" s="18" t="inlineStr">
         <is>
-          <t>Kylskåpsspärrarna 2-pack husvagn</t>
+          <t>Vindavvisarna till Ducato-hytten, par</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $16.05. Vår räkning: landad ca 232 kr, tänkt butikspris 499 kr. Originaltitel: Kylskåpsspärrarna 2-pack husvagn</t>
+          <t>AliExpress: US $24.09. Vår räkning: landad ca 348 kr, tänkt butikspris 649 kr. Originaltitel: Vindavvisarna till Ducato-hytten, par</t>
         </is>
       </c>
       <c r="H37" s="13" t="n"/>
@@ -2814,7 +2839,7 @@
       <c r="M37" s="14" t="n"/>
       <c r="N37" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010339744458.html</t>
+          <t>https://www.aliexpress.com/item/1005012880104542.html</t>
         </is>
       </c>
       <c r="Q37" s="18" t="n"/>
@@ -2964,12 +2989,12 @@
       <c r="A41" s="10" t="n"/>
       <c r="D41" s="18" t="inlineStr">
         <is>
-          <t>Överskåpsspärrarna 3-pack (elastisk lina)</t>
+          <t>Kylskåpsspärrarna 2-pack husvagn</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $6.39. Vår räkning: landad ca 277 kr, tänkt butikspris 499 kr. Originaltitel: Överskåpsspärrarna 3-pack (elastisk lina)</t>
+          <t>AliExpress: US $16.05. Vår räkning: landad ca 232 kr, tänkt butikspris 499 kr. Originaltitel: Kylskåpsspärrarna 2-pack husvagn</t>
         </is>
       </c>
       <c r="H41" s="13" t="n"/>
@@ -2984,7 +3009,7 @@
       <c r="M41" s="14" t="n"/>
       <c r="N41" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012201958598.html</t>
+          <t>https://www.aliexpress.com/item/1005010339744458.html</t>
         </is>
       </c>
       <c r="Q41" s="18" t="n"/>
@@ -3134,12 +3159,12 @@
       <c r="A45" s="10" t="n"/>
       <c r="D45" s="18" t="inlineStr">
         <is>
-          <t>Dörrhaspen med dolt hänglås</t>
+          <t>Överskåpsspärrarna 3-pack (elastisk lina)</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $18.36. Vår räkning: landad ca 265 kr, tänkt butikspris 599 kr. Originaltitel: Dörrhaspen med dolt hänglås</t>
+          <t>AliExpress: US $6.39. Vår räkning: landad ca 277 kr, tänkt butikspris 499 kr. Originaltitel: Överskåpsspärrarna 3-pack (elastisk lina)</t>
         </is>
       </c>
       <c r="H45" s="13" t="n"/>
@@ -3154,7 +3179,7 @@
       <c r="M45" s="14" t="n"/>
       <c r="N45" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010518810434.html</t>
+          <t>https://www.aliexpress.com/item/1005012201958598.html</t>
         </is>
       </c>
       <c r="Q45" s="18" t="n"/>
@@ -3304,12 +3329,12 @@
       <c r="A49" s="10" t="n"/>
       <c r="D49" s="18" t="inlineStr">
         <is>
-          <t>Takrännans droppnäsor, 4-pack</t>
+          <t>Dörrhaspen med dolt hänglås</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $11.55. Vår räkning: landad ca 167 kr, tänkt butikspris 429 kr. Originaltitel: Takrännans droppnäsor, 4-pack</t>
+          <t>AliExpress: US $18.36. Vår räkning: landad ca 265 kr, tänkt butikspris 599 kr. Originaltitel: Dörrhaspen med dolt hänglås</t>
         </is>
       </c>
       <c r="H49" s="13" t="n"/>
@@ -3324,7 +3349,7 @@
       <c r="M49" s="14" t="n"/>
       <c r="N49" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005013242934199.html</t>
+          <t>https://www.aliexpress.com/item/1005010518810434.html</t>
         </is>
       </c>
       <c r="Q49" s="18" t="n"/>
@@ -3474,12 +3499,12 @@
       <c r="A53" s="10" t="n"/>
       <c r="D53" s="18" t="inlineStr">
         <is>
-          <t>Droppkantslisten mot svarta ränder, 2 × 3 m</t>
+          <t>Takrännans droppnäsor, 4-pack</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $12.06. Vår räkning: landad ca 349 kr, tänkt butikspris 699 kr. Originaltitel: Droppkantslisten mot svarta ränder, 2 × 3 m</t>
+          <t>AliExpress: US $11.55. Vår räkning: landad ca 167 kr, tänkt butikspris 429 kr. Originaltitel: Takrännans droppnäsor, 4-pack</t>
         </is>
       </c>
       <c r="H53" s="13" t="n"/>
@@ -3494,7 +3519,7 @@
       <c r="M53" s="14" t="n"/>
       <c r="N53" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005009863338287.html</t>
+          <t>https://www.aliexpress.com/item/1005013242934199.html</t>
         </is>
       </c>
       <c r="Q53" s="18" t="n"/>
@@ -3644,12 +3669,12 @@
       <c r="A57" s="10" t="n"/>
       <c r="D57" s="18" t="inlineStr">
         <is>
-          <t>Hjullåset för husvagn (Milenco-kopia)</t>
+          <t>Droppkantslisten mot svarta ränder, 2 × 3 m</t>
         </is>
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $34.56. Vår räkning: landad ca 500 kr, tänkt butikspris 949 kr. Originaltitel: Hjullåset för husvagn (Milenco-kopia)</t>
+          <t>AliExpress: US $12.06. Vår räkning: landad ca 349 kr, tänkt butikspris 699 kr. Originaltitel: Droppkantslisten mot svarta ränder, 2 × 3 m</t>
         </is>
       </c>
       <c r="H57" s="13" t="n"/>
@@ -3664,7 +3689,7 @@
       <c r="M57" s="14" t="n"/>
       <c r="N57" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012671051312.html</t>
+          <t>https://www.aliexpress.com/item/1005009863338287.html</t>
         </is>
       </c>
       <c r="Q57" s="18" t="n"/>
@@ -3814,12 +3839,12 @@
       <c r="A61" s="10" t="n"/>
       <c r="D61" s="18" t="inlineStr">
         <is>
-          <t>Fönsterspärrarna Seitz/Dometic, 3 par</t>
+          <t>Hjullåset för husvagn (Milenco-kopia)</t>
         </is>
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $2.26. Vår räkning: landad ca 98 kr, tänkt butikspris 349 kr. Originaltitel: Fönsterspärrarna Seitz/Dometic, 3 par</t>
+          <t>AliExpress: US $34.56. Vår räkning: landad ca 500 kr, tänkt butikspris 949 kr. Originaltitel: Hjullåset för husvagn (Milenco-kopia)</t>
         </is>
       </c>
       <c r="H61" s="13" t="n"/>
@@ -3834,7 +3859,7 @@
       <c r="M61" s="14" t="n"/>
       <c r="N61" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012010863972.html</t>
+          <t>https://www.aliexpress.com/item/1005012671051312.html</t>
         </is>
       </c>
       <c r="Q61" s="18" t="n"/>
@@ -3984,12 +4009,12 @@
       <c r="A65" s="10" t="n"/>
       <c r="D65" s="18" t="inlineStr">
         <is>
-          <t>Vattentankens värmedyna 12 V</t>
+          <t>Fönsterspärrarna Seitz/Dometic, 3 par</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $13.65. Vår räkning: landad ca 198 kr, tänkt butikspris 479 kr. Originaltitel: Vattentankens värmedyna 12 V</t>
+          <t>AliExpress: US $2.26. Vår räkning: landad ca 98 kr, tänkt butikspris 349 kr. Originaltitel: Fönsterspärrarna Seitz/Dometic, 3 par</t>
         </is>
       </c>
       <c r="H65" s="13" t="n"/>
@@ -4004,7 +4029,7 @@
       <c r="M65" s="14" t="n"/>
       <c r="N65" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005007345717544.html</t>
+          <t>https://www.aliexpress.com/item/1005012010863972.html</t>
         </is>
       </c>
       <c r="Q65" s="18" t="n"/>
@@ -4150,10 +4175,176 @@
       <c r="AT68" s="35" t="n"/>
       <c r="AU68" s="35" t="n"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" s="71"/>
-    <row r="70" ht="15.75" customHeight="1" s="71"/>
-    <row r="71" ht="15.75" customHeight="1" s="71"/>
-    <row r="72" ht="15.75" customHeight="1" s="71"/>
+    <row r="69" ht="45" customHeight="1" s="71">
+      <c r="A69" s="10" t="n"/>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>Vattentankens värmedyna 12 V</t>
+        </is>
+      </c>
+      <c r="E69" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $13.65. Vår räkning: landad ca 198 kr, tänkt butikspris 479 kr. Originaltitel: Vattentankens värmedyna 12 V</t>
+        </is>
+      </c>
+      <c r="H69" s="13" t="n"/>
+      <c r="I69" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J69" s="15" t="n"/>
+      <c r="K69" s="15" t="n"/>
+      <c r="L69" s="16" t="n"/>
+      <c r="M69" s="14" t="n"/>
+      <c r="N69" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005007345717544.html</t>
+        </is>
+      </c>
+      <c r="Q69" s="18" t="n"/>
+      <c r="R69" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S69" s="15" t="n"/>
+      <c r="T69" s="15" t="n"/>
+      <c r="U69" s="16" t="n"/>
+      <c r="V69" s="48" t="n"/>
+      <c r="W69" s="48" t="n"/>
+      <c r="X69" s="21" t="n"/>
+      <c r="Y69" s="15" t="n"/>
+      <c r="Z69" s="15" t="n"/>
+      <c r="AA69" s="16" t="n"/>
+      <c r="AB69" s="48" t="n"/>
+      <c r="AC69" s="48" t="n"/>
+      <c r="AD69" s="22" t="n"/>
+      <c r="AE69" s="15" t="n"/>
+      <c r="AF69" s="15" t="n"/>
+      <c r="AG69" s="16" t="n"/>
+      <c r="AH69" s="48" t="n"/>
+      <c r="AI69" s="48" t="n"/>
+      <c r="AJ69" s="23" t="n"/>
+      <c r="AK69" s="15" t="n"/>
+      <c r="AL69" s="15" t="n"/>
+      <c r="AM69" s="16" t="n"/>
+      <c r="AN69" s="25" t="n"/>
+      <c r="AO69" s="48" t="n"/>
+      <c r="AP69" s="23" t="n"/>
+      <c r="AQ69" s="15" t="n"/>
+      <c r="AR69" s="15" t="n"/>
+      <c r="AS69" s="16" t="n"/>
+      <c r="AT69" s="25" t="n"/>
+      <c r="AU69" s="26" t="n"/>
+    </row>
+    <row r="70" ht="45" customHeight="1" s="71">
+      <c r="D70" s="18" t="n"/>
+      <c r="J70" s="15" t="n"/>
+      <c r="K70" s="15" t="n"/>
+      <c r="L70" s="16" t="n"/>
+      <c r="R70" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S70" s="15" t="n"/>
+      <c r="T70" s="15" t="n"/>
+      <c r="U70" s="16" t="n"/>
+      <c r="X70" s="21" t="n"/>
+      <c r="Y70" s="15" t="n"/>
+      <c r="Z70" s="15" t="n"/>
+      <c r="AA70" s="16" t="n"/>
+      <c r="AD70" s="22" t="n"/>
+      <c r="AE70" s="15" t="n"/>
+      <c r="AF70" s="15" t="n"/>
+      <c r="AG70" s="16" t="n"/>
+      <c r="AH70" s="48" t="n"/>
+      <c r="AI70" s="48" t="n"/>
+      <c r="AJ70" s="23" t="n"/>
+      <c r="AK70" s="15" t="n"/>
+      <c r="AL70" s="15" t="n"/>
+      <c r="AM70" s="16" t="n"/>
+      <c r="AP70" s="23" t="n"/>
+      <c r="AQ70" s="15" t="n"/>
+      <c r="AR70" s="15" t="n"/>
+      <c r="AS70" s="16" t="n"/>
+    </row>
+    <row r="71" ht="45" customHeight="1" s="71">
+      <c r="D71" s="18" t="n"/>
+      <c r="J71" s="15" t="n"/>
+      <c r="K71" s="15" t="n"/>
+      <c r="L71" s="16" t="n"/>
+      <c r="R71" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S71" s="15" t="n"/>
+      <c r="T71" s="15" t="n"/>
+      <c r="U71" s="16" t="n"/>
+      <c r="X71" s="21" t="n"/>
+      <c r="Y71" s="15" t="n"/>
+      <c r="Z71" s="15" t="n"/>
+      <c r="AA71" s="16" t="n"/>
+      <c r="AD71" s="22" t="n"/>
+      <c r="AE71" s="15" t="n"/>
+      <c r="AF71" s="15" t="n"/>
+      <c r="AG71" s="16" t="n"/>
+      <c r="AH71" s="48" t="n"/>
+      <c r="AI71" s="48" t="n"/>
+      <c r="AJ71" s="23" t="n"/>
+      <c r="AK71" s="15" t="n"/>
+      <c r="AL71" s="15" t="n"/>
+      <c r="AM71" s="16" t="n"/>
+      <c r="AP71" s="23" t="n"/>
+      <c r="AQ71" s="15" t="n"/>
+      <c r="AR71" s="15" t="n"/>
+      <c r="AS71" s="16" t="n"/>
+    </row>
+    <row r="72" ht="6.75" customHeight="1" s="71">
+      <c r="A72" s="27" t="n"/>
+      <c r="B72" s="27" t="n"/>
+      <c r="C72" s="27" t="n"/>
+      <c r="D72" s="27" t="n"/>
+      <c r="E72" s="27" t="n"/>
+      <c r="F72" s="27" t="n"/>
+      <c r="G72" s="27" t="n"/>
+      <c r="H72" s="35" t="n"/>
+      <c r="I72" s="35" t="n"/>
+      <c r="J72" s="36" t="n"/>
+      <c r="K72" s="36" t="n"/>
+      <c r="L72" s="36" t="n"/>
+      <c r="M72" s="35" t="n"/>
+      <c r="N72" s="30" t="n"/>
+      <c r="O72" s="30" t="n"/>
+      <c r="P72" s="30" t="n"/>
+      <c r="Q72" s="30" t="n"/>
+      <c r="R72" s="35" t="n"/>
+      <c r="S72" s="35" t="n"/>
+      <c r="T72" s="35" t="n"/>
+      <c r="U72" s="35" t="n"/>
+      <c r="V72" s="35" t="n"/>
+      <c r="W72" s="35" t="n"/>
+      <c r="X72" s="31" t="n"/>
+      <c r="Y72" s="35" t="n"/>
+      <c r="Z72" s="35" t="n"/>
+      <c r="AA72" s="36" t="n"/>
+      <c r="AB72" s="35" t="n"/>
+      <c r="AC72" s="35" t="n"/>
+      <c r="AD72" s="32" t="n"/>
+      <c r="AE72" s="35" t="n"/>
+      <c r="AF72" s="35" t="n"/>
+      <c r="AG72" s="36" t="n"/>
+      <c r="AH72" s="35" t="n"/>
+      <c r="AI72" s="35" t="n"/>
+      <c r="AJ72" s="34" t="n"/>
+      <c r="AK72" s="35" t="n"/>
+      <c r="AL72" s="35" t="n"/>
+      <c r="AM72" s="36" t="n"/>
+      <c r="AN72" s="35" t="n"/>
+      <c r="AO72" s="35" t="n"/>
+      <c r="AP72" s="34" t="n"/>
+      <c r="AQ72" s="35" t="n"/>
+      <c r="AR72" s="35" t="n"/>
+      <c r="AS72" s="36" t="n"/>
+      <c r="AT72" s="35" t="n"/>
+      <c r="AU72" s="35" t="n"/>
+    </row>
     <row r="73" ht="15.75" customHeight="1" s="71"/>
     <row r="74" ht="15.75" customHeight="1" s="71"/>
     <row r="75" ht="15.75" customHeight="1" s="71"/>
@@ -5083,12 +5274,14 @@
     <row r="999" ht="15.75" customHeight="1" s="71"/>
     <row r="1000" ht="15.75" customHeight="1" s="71"/>
   </sheetData>
-  <mergeCells count="129">
+  <mergeCells count="136">
     <mergeCell ref="E5:G7"/>
     <mergeCell ref="H17:H19"/>
+    <mergeCell ref="H69:H71"/>
     <mergeCell ref="M21:M23"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="M57:M59"/>
+    <mergeCell ref="E69:G71"/>
     <mergeCell ref="N5:P7"/>
     <mergeCell ref="M41:M43"/>
     <mergeCell ref="N33:P35"/>
@@ -5112,6 +5305,7 @@
     <mergeCell ref="AP3:AU3"/>
     <mergeCell ref="H21:H23"/>
     <mergeCell ref="I53:I55"/>
+    <mergeCell ref="M69:M71"/>
     <mergeCell ref="M25:M27"/>
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="M61:M63"/>
@@ -5120,6 +5314,7 @@
     <mergeCell ref="H57:H59"/>
     <mergeCell ref="Q9:Q11"/>
     <mergeCell ref="M45:M47"/>
+    <mergeCell ref="Q69:Q71"/>
     <mergeCell ref="I29:I31"/>
     <mergeCell ref="I13:I15"/>
     <mergeCell ref="E61:G63"/>
@@ -5145,6 +5340,7 @@
     <mergeCell ref="N53:P55"/>
     <mergeCell ref="I33:I35"/>
     <mergeCell ref="H61:H63"/>
+    <mergeCell ref="A69:C71"/>
     <mergeCell ref="I5:I7"/>
     <mergeCell ref="Q65:Q67"/>
     <mergeCell ref="I17:I19"/>
@@ -5163,6 +5359,7 @@
     <mergeCell ref="Q45:Q47"/>
     <mergeCell ref="Q17:Q19"/>
     <mergeCell ref="E9:G11"/>
+    <mergeCell ref="I69:I71"/>
     <mergeCell ref="M3:M4"/>
     <mergeCell ref="Q13:Q15"/>
     <mergeCell ref="N13:P15"/>
@@ -5198,6 +5395,7 @@
     <mergeCell ref="N29:P31"/>
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="A33:C35"/>
+    <mergeCell ref="N69:P71"/>
     <mergeCell ref="Q53:Q55"/>
     <mergeCell ref="E41:G43"/>
     <mergeCell ref="I45:I47"/>

</xml_diff>

<commit_message>
produktjakt Carashell: hjulöverdragen 4-pack döpta om och först på sidan (v33), ark ombyggt
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jBJVGuyny8S3j2XPSM26Z
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-29-carashell/Leverantorsoffert-2026-09-29-carashell.xlsx
+++ b/produktjakt/korningar/2026-09-29-carashell/Leverantorsoffert-2026-09-29-carashell.xlsx
@@ -566,7 +566,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2133600" cy="1600200"/>
+    <ext cx="1600200" cy="1600200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -591,7 +591,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1600200" cy="1600200"/>
+    <ext cx="2133600" cy="1600200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -1459,12 +1459,12 @@
       <c r="A5" s="10" t="n"/>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Gnagarstaketet runt husbilen, 304-nät</t>
+          <t>Hjulöverdragen 4-pack — ett per hjul, silver</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $28.09. Vår räkning: landad ca 406 kr, tänkt butikspris 979 kr. Originaltitel: Gnagarstaketet runt husbilen, 304-nät</t>
+          <t>AliExpress: US $24.49. Vår räkning: landad ca 355 kr, tänkt butikspris 599 kr. Originaltitel: Hjulskydden 4-pack, silver 19–36 tum</t>
         </is>
       </c>
       <c r="H5" s="13" t="n"/>
@@ -1479,7 +1479,7 @@
       <c r="M5" s="14" t="n"/>
       <c r="N5" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012197754256.html</t>
+          <t>https://www.aliexpress.com/item/1005005932851254.html</t>
         </is>
       </c>
       <c r="Q5" s="18" t="n"/>
@@ -1629,12 +1629,12 @@
       <c r="A9" s="10" t="n"/>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Hyttavskiljaren — termogardin Ducato</t>
+          <t>Gnagarstaketet runt husbilen, 304-nät</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $33.49. Vår räkning: landad ca 484 kr, tänkt butikspris 1199 kr. Originaltitel: Hyttavskiljaren — termogardin Ducato</t>
+          <t>AliExpress: US $28.09. Vår räkning: landad ca 406 kr, tänkt butikspris 979 kr. Originaltitel: Gnagarstaketet runt husbilen, 304-nät</t>
         </is>
       </c>
       <c r="H9" s="13" t="n"/>
@@ -1649,7 +1649,7 @@
       <c r="M9" s="14" t="n"/>
       <c r="N9" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010501442950.html</t>
+          <t>https://www.aliexpress.com/item/1005012197754256.html</t>
         </is>
       </c>
       <c r="Q9" s="18" t="n"/>
@@ -1799,12 +1799,12 @@
       <c r="A13" s="10" t="n"/>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Midi Heki-huven hagel &amp; termo</t>
+          <t>Hyttavskiljaren — termogardin Ducato</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $12.15. Vår räkning: landad ca 176 kr, tänkt butikspris 599 kr. Originaltitel: Midi Heki-huven hagel &amp; termo</t>
+          <t>AliExpress: US $33.49. Vår räkning: landad ca 484 kr, tänkt butikspris 1199 kr. Originaltitel: Hyttavskiljaren — termogardin Ducato</t>
         </is>
       </c>
       <c r="H13" s="13" t="n"/>
@@ -1819,7 +1819,7 @@
       <c r="M13" s="14" t="n"/>
       <c r="N13" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005013036934132.html</t>
+          <t>https://www.aliexpress.com/item/1005010501442950.html</t>
         </is>
       </c>
       <c r="Q13" s="18" t="n"/>
@@ -1969,12 +1969,12 @@
       <c r="A17" s="10" t="n"/>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Vinterkjolen 7 m med hjulhuskappor</t>
+          <t>Midi Heki-huven hagel &amp; termo</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $17.09. Vår räkning: landad ca 247 kr, tänkt butikspris 599 kr. Originaltitel: Vinterkjolen 7 m med hjulhuskappor</t>
+          <t>AliExpress: US $12.15. Vår räkning: landad ca 176 kr, tänkt butikspris 599 kr. Originaltitel: Midi Heki-huven hagel &amp; termo</t>
         </is>
       </c>
       <c r="H17" s="13" t="n"/>
@@ -1989,7 +1989,7 @@
       <c r="M17" s="14" t="n"/>
       <c r="N17" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005009861098478.html</t>
+          <t>https://www.aliexpress.com/item/1005013036934132.html</t>
         </is>
       </c>
       <c r="Q17" s="18" t="n"/>
@@ -2139,12 +2139,12 @@
       <c r="A21" s="10" t="n"/>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>Skjutdörrsgardinen Ducato, magnetisk</t>
+          <t>Vinterkjolen 7 m med hjulhuskappor</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $23.09. Vår räkning: landad ca 334 kr, tänkt butikspris 999 kr. Originaltitel: Skjutdörrsgardinen Ducato, magnetisk</t>
+          <t>AliExpress: US $17.09. Vår räkning: landad ca 247 kr, tänkt butikspris 599 kr. Originaltitel: Vinterkjolen 7 m med hjulhuskappor</t>
         </is>
       </c>
       <c r="H21" s="13" t="n"/>
@@ -2159,7 +2159,7 @@
       <c r="M21" s="14" t="n"/>
       <c r="N21" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010001321489.html</t>
+          <t>https://www.aliexpress.com/item/1005009861098478.html</t>
         </is>
       </c>
       <c r="Q21" s="18" t="n"/>
@@ -2309,12 +2309,12 @@
       <c r="A25" s="10" t="n"/>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>Hjulskydden 4-pack, silver 19–36 tum</t>
+          <t>Skjutdörrsgardinen Ducato, magnetisk</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $24.49. Vår räkning: landad ca 355 kr, tänkt butikspris 599 kr. Originaltitel: Hjulskydden 4-pack, silver 19–36 tum</t>
+          <t>AliExpress: US $23.09. Vår räkning: landad ca 334 kr, tänkt butikspris 999 kr. Originaltitel: Skjutdörrsgardinen Ducato, magnetisk</t>
         </is>
       </c>
       <c r="H25" s="13" t="n"/>
@@ -2329,7 +2329,7 @@
       <c r="M25" s="14" t="n"/>
       <c r="N25" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005005932851254.html</t>
+          <t>https://www.aliexpress.com/item/1005010001321489.html</t>
         </is>
       </c>
       <c r="Q25" s="18" t="n"/>

</xml_diff>